<commit_message>
Update playwin translations Excel file
</commit_message>
<xml_diff>
--- a/playwin/locales-excel/playwin_translations.xlsx
+++ b/playwin/locales-excel/playwin_translations.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G527"/>
+  <dimension ref="A1:G528"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10461,27 +10461,27 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>A minimum deposit of {{min}} is required</t>
+          <t>A minimum deposit of ₹{{min}} is required</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>ઓછામાં ઓછી {{min}} ની ડિપૉઝિટ જરૂરી છે</t>
+          <t>ઓછામાં ઓછી ₹{{min}} ની ડિપૉઝિટ જરૂરી છે</t>
         </is>
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>न्यूनतम {{min}} की जमा आवश्यक है</t>
+          <t>न्यूनतम ₹{{min}} की जमा आवश्यक है</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>குறைந்தது {{min}} வைப்பு தேவை</t>
+          <t>குறைந்தது ₹{{min}} வைப்பு தேவை</t>
         </is>
       </c>
       <c r="G272" t="inlineStr">
         <is>
-          <t>కనీసం {{min}} డిపాజిట్ అవసరం</t>
+          <t>కనీసం ₹{{min}} డిపాజిట్ అవసరం</t>
         </is>
       </c>
     </row>
@@ -18929,32 +18929,32 @@
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>transactionTable.dateSelector.lastMonth</t>
+          <t>transactionTable.dateSelector.custom</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>Last Month</t>
+          <t>Custom Range</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
         <is>
-          <t>ગત મહિને</t>
+          <t>કસ્ટમ રેંજ</t>
         </is>
       </c>
       <c r="E501" t="inlineStr">
         <is>
-          <t>पिछले महीने</t>
+          <t>कस्टम रेंज</t>
         </is>
       </c>
       <c r="F501" t="inlineStr">
         <is>
-          <t>கடந்த மாதம்</t>
+          <t>தனிப்பயன் வரம்பு</t>
         </is>
       </c>
       <c r="G501" t="inlineStr">
         <is>
-          <t>గత నెల</t>
+          <t>కస్టమ్ రేంజ్</t>
         </is>
       </c>
     </row>
@@ -18966,32 +18966,32 @@
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>transactionTable.dateSelector.lastWeek</t>
+          <t>transactionTable.dateSelector.lastMonth</t>
         </is>
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>Last Week</t>
+          <t>Last Month</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
         <is>
-          <t>ગત અઠવાડિયે</t>
+          <t>ગત મહિને</t>
         </is>
       </c>
       <c r="E502" t="inlineStr">
         <is>
-          <t>पिछले सप्ताह</t>
+          <t>पिछले महीने</t>
         </is>
       </c>
       <c r="F502" t="inlineStr">
         <is>
-          <t>கடந்த வாரம்</t>
+          <t>கடந்த மாதம்</t>
         </is>
       </c>
       <c r="G502" t="inlineStr">
         <is>
-          <t>గత వారం</t>
+          <t>గత నెల</t>
         </is>
       </c>
     </row>
@@ -19003,32 +19003,32 @@
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>transactionTable.dateSelector.thisMonth</t>
+          <t>transactionTable.dateSelector.lastWeek</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>This Month</t>
+          <t>Last Week</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
         <is>
-          <t>આ મહિને</t>
+          <t>ગત અઠવાડિયે</t>
         </is>
       </c>
       <c r="E503" t="inlineStr">
         <is>
-          <t>इस महीने</t>
+          <t>पिछले सप्ताह</t>
         </is>
       </c>
       <c r="F503" t="inlineStr">
         <is>
-          <t>இந்த மாதம்</t>
+          <t>கடந்த வாரம்</t>
         </is>
       </c>
       <c r="G503" t="inlineStr">
         <is>
-          <t>ఈ నెల</t>
+          <t>గత వారం</t>
         </is>
       </c>
     </row>
@@ -19040,32 +19040,32 @@
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>transactionTable.dateSelector.thisWeek</t>
+          <t>transactionTable.dateSelector.thisMonth</t>
         </is>
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>This Week</t>
+          <t>This Month</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
         <is>
-          <t>આ અઠવાડિયે</t>
+          <t>આ મહિને</t>
         </is>
       </c>
       <c r="E504" t="inlineStr">
         <is>
-          <t>इस सप्ताह</t>
+          <t>इस महीने</t>
         </is>
       </c>
       <c r="F504" t="inlineStr">
         <is>
-          <t>இந்த வாரம்</t>
+          <t>இந்த மாதம்</t>
         </is>
       </c>
       <c r="G504" t="inlineStr">
         <is>
-          <t>ఈ వారం</t>
+          <t>ఈ నెల</t>
         </is>
       </c>
     </row>
@@ -19077,32 +19077,32 @@
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>transactionTable.dateSelector.today</t>
+          <t>transactionTable.dateSelector.thisWeek</t>
         </is>
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>Today</t>
+          <t>This Week</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
         <is>
-          <t>આજ</t>
+          <t>આ અઠવાડિયે</t>
         </is>
       </c>
       <c r="E505" t="inlineStr">
         <is>
-          <t>आज</t>
+          <t>इस सप्ताह</t>
         </is>
       </c>
       <c r="F505" t="inlineStr">
         <is>
-          <t>இன்று</t>
+          <t>இந்த வாரம்</t>
         </is>
       </c>
       <c r="G505" t="inlineStr">
         <is>
-          <t>నేడు</t>
+          <t>ఈ వారం</t>
         </is>
       </c>
     </row>
@@ -19114,32 +19114,32 @@
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>transactionTable.dateSelector.yesterday</t>
+          <t>transactionTable.dateSelector.today</t>
         </is>
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>Yesterday</t>
+          <t>Today</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
         <is>
-          <t>ગઈ કાલ</t>
+          <t>આજ</t>
         </is>
       </c>
       <c r="E506" t="inlineStr">
         <is>
-          <t>कल</t>
+          <t>आज</t>
         </is>
       </c>
       <c r="F506" t="inlineStr">
         <is>
-          <t>நேற்று</t>
+          <t>இன்று</t>
         </is>
       </c>
       <c r="G506" t="inlineStr">
         <is>
-          <t>నిన్న</t>
+          <t>నేడు</t>
         </is>
       </c>
     </row>
@@ -19151,32 +19151,32 @@
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>transactionTable.pagination.next</t>
+          <t>transactionTable.dateSelector.yesterday</t>
         </is>
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Yesterday</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
         <is>
-          <t>આગળ</t>
+          <t>ગઈ કાલ</t>
         </is>
       </c>
       <c r="E507" t="inlineStr">
         <is>
-          <t>अगला</t>
+          <t>कल</t>
         </is>
       </c>
       <c r="F507" t="inlineStr">
         <is>
-          <t>அடுத்த</t>
+          <t>நேற்று</t>
         </is>
       </c>
       <c r="G507" t="inlineStr">
         <is>
-          <t>తదుపరి</t>
+          <t>నిన్న</t>
         </is>
       </c>
     </row>
@@ -19188,32 +19188,32 @@
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>transactionTable.pagination.prev</t>
+          <t>transactionTable.pagination.next</t>
         </is>
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Next</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
         <is>
-          <t>પહેલા</t>
+          <t>આગળ</t>
         </is>
       </c>
       <c r="E508" t="inlineStr">
         <is>
-          <t>पिछला</t>
+          <t>अगला</t>
         </is>
       </c>
       <c r="F508" t="inlineStr">
         <is>
-          <t>முந்தைய</t>
+          <t>அடுத்த</t>
         </is>
       </c>
       <c r="G508" t="inlineStr">
         <is>
-          <t>మునుపటి</t>
+          <t>తదుపరి</t>
         </is>
       </c>
     </row>
@@ -19225,69 +19225,69 @@
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>transactionTable.pagination.rowsPerPage</t>
+          <t>transactionTable.pagination.prev</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>Rows per page:</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
         <is>
-          <t>પ્રતિ પૃષ્ઠ પ્રવૃત્તિઓ:</t>
+          <t>પહેલા</t>
         </is>
       </c>
       <c r="E509" t="inlineStr">
         <is>
-          <t>प्रति पृष्ठ पंक्तियां:</t>
+          <t>पिछला</t>
         </is>
       </c>
       <c r="F509" t="inlineStr">
         <is>
-          <t>பக்கத்திற்கு வரிசைகள்:</t>
+          <t>முந்தைய</t>
         </is>
       </c>
       <c r="G509" t="inlineStr">
         <is>
-          <t>పేజీకి వరుసలు:</t>
+          <t>మునుపటి</t>
         </is>
       </c>
     </row>
     <row r="510">
       <c r="A510" t="inlineStr">
         <is>
-          <t>wallet</t>
+          <t>transactionHistory</t>
         </is>
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>moneySuffix</t>
+          <t>transactionTable.pagination.rowsPerPage</t>
         </is>
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>{{wallet}} Money</t>
+          <t>Rows per page:</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
         <is>
-          <t>{{wallet}} મની</t>
+          <t>પ્રતિ પૃષ્ઠ પ્રવૃત્તિઓ:</t>
         </is>
       </c>
       <c r="E510" t="inlineStr">
         <is>
-          <t>{{wallet}} पैसे</t>
+          <t>प्रति पृष्ठ पंक्तियां:</t>
         </is>
       </c>
       <c r="F510" t="inlineStr">
         <is>
-          <t>{{wallet}} பணம்</t>
+          <t>பக்கத்திற்கு வரிசைகள்:</t>
         </is>
       </c>
       <c r="G510" t="inlineStr">
         <is>
-          <t>{{wallet}} డబ్బు</t>
+          <t>పేజీకి వరుసలు:</t>
         </is>
       </c>
     </row>
@@ -19299,32 +19299,32 @@
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>realMoney</t>
+          <t>moneySuffix</t>
         </is>
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>Real Money ₹ {{amount}}</t>
+          <t>{{wallet}} Money</t>
         </is>
       </c>
       <c r="D511" t="inlineStr">
         <is>
-          <t>રિઅલ મની ₹ {{amount}}</t>
+          <t>{{wallet}} મની</t>
         </is>
       </c>
       <c r="E511" t="inlineStr">
         <is>
-          <t>असली पैसे ₹ {{amount}}</t>
+          <t>{{wallet}} पैसे</t>
         </is>
       </c>
       <c r="F511" t="inlineStr">
         <is>
-          <t>உண்மையான பணம் ₹ {{amount}}</t>
+          <t>{{wallet}} பணம்</t>
         </is>
       </c>
       <c r="G511" t="inlineStr">
         <is>
-          <t>నిజమైన డబ్బు ₹ {{amount}}</t>
+          <t>{{wallet}} డబ్బు</t>
         </is>
       </c>
     </row>
@@ -19336,32 +19336,32 @@
       </c>
       <c r="B512" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>realMoney</t>
         </is>
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>Wallet</t>
+          <t>Real Money ₹ {{amount}}</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
         <is>
-          <t>વૉલેટ</t>
+          <t>રિઅલ મની ₹ {{amount}}</t>
         </is>
       </c>
       <c r="E512" t="inlineStr">
         <is>
-          <t>वॉलेट</t>
+          <t>असली पैसे ₹ {{amount}}</t>
         </is>
       </c>
       <c r="F512" t="inlineStr">
         <is>
-          <t>பணப்பை</t>
+          <t>உண்மையான பணம் ₹ {{amount}}</t>
         </is>
       </c>
       <c r="G512" t="inlineStr">
         <is>
-          <t>వాలెట్</t>
+          <t>నిజమైన డబ్బు ₹ {{amount}}</t>
         </is>
       </c>
     </row>
@@ -19373,69 +19373,69 @@
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>withdrawableMoney</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>Withdrawable Money ₹ {{amount}}</t>
+          <t>Wallet</t>
         </is>
       </c>
       <c r="D513" t="inlineStr">
         <is>
-          <t>ઉપાડ યોગ્ય મની ₹ {{amount}}</t>
+          <t>વૉલેટ</t>
         </is>
       </c>
       <c r="E513" t="inlineStr">
         <is>
-          <t>निकासी योग्य पैसे ₹ {{amount}}</t>
+          <t>वॉलेट</t>
         </is>
       </c>
       <c r="F513" t="inlineStr">
         <is>
-          <t>திரும்பப் பெறக்கூடிய பணம் ₹ {{amount}}</t>
+          <t>பணப்பை</t>
         </is>
       </c>
       <c r="G513" t="inlineStr">
         <is>
-          <t>ఉపసంహరించదగిన డబ్బు ₹ {{amount}}</t>
+          <t>వాలెట్</t>
         </is>
       </c>
     </row>
     <row r="514">
       <c r="A514" t="inlineStr">
         <is>
-          <t>withdraw</t>
+          <t>wallet</t>
         </is>
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>enterAmountPlaceholder</t>
+          <t>withdrawableMoney</t>
         </is>
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>Enter Amount</t>
+          <t>Withdrawable Money ₹ {{amount}}</t>
         </is>
       </c>
       <c r="D514" t="inlineStr">
         <is>
-          <t>રકમ દાખલ કરો</t>
+          <t>ઉપાડ યોગ્ય મની ₹ {{amount}}</t>
         </is>
       </c>
       <c r="E514" t="inlineStr">
         <is>
-          <t>राशि दर्ज करें</t>
+          <t>निकासी योग्य पैसे ₹ {{amount}}</t>
         </is>
       </c>
       <c r="F514" t="inlineStr">
         <is>
-          <t>தொகையை உள்ளிடவும்</t>
+          <t>திரும்பப் பெறக்கூடிய பணம் ₹ {{amount}}</t>
         </is>
       </c>
       <c r="G514" t="inlineStr">
         <is>
-          <t>మొత్తాన్ని నమోదు చేయండి</t>
+          <t>ఉపసంహరించదగిన డబ్బు ₹ {{amount}}</t>
         </is>
       </c>
     </row>
@@ -19447,32 +19447,32 @@
       </c>
       <c r="B515" t="inlineStr">
         <is>
-          <t>selectBankPlaceholder</t>
+          <t>enterAmountPlaceholder</t>
         </is>
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>Select Bank Account</t>
+          <t>Enter Amount</t>
         </is>
       </c>
       <c r="D515" t="inlineStr">
         <is>
-          <t>બૅન્ક ખાતું પસંદ કરો</t>
+          <t>રકમ દાખલ કરો</t>
         </is>
       </c>
       <c r="E515" t="inlineStr">
         <is>
-          <t>बैंक खाता चुनें</t>
+          <t>राशि दर्ज करें</t>
         </is>
       </c>
       <c r="F515" t="inlineStr">
         <is>
-          <t>வங்கி கணக்கை தேர்வு செய்யவும்</t>
+          <t>தொகையை உள்ளிடவும்</t>
         </is>
       </c>
       <c r="G515" t="inlineStr">
         <is>
-          <t>బ్యాంకు ఖాతాను ఎంచుకోండి</t>
+          <t>మొత్తాన్ని నమోదు చేయండి</t>
         </is>
       </c>
     </row>
@@ -19484,32 +19484,32 @@
       </c>
       <c r="B516" t="inlineStr">
         <is>
-          <t>submit</t>
+          <t>selectBankPlaceholder</t>
         </is>
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>Withdraw</t>
+          <t>Select Bank Account</t>
         </is>
       </c>
       <c r="D516" t="inlineStr">
         <is>
-          <t>ઉપાડ કરો</t>
+          <t>બૅન્ક ખાતું પસંદ કરો</t>
         </is>
       </c>
       <c r="E516" t="inlineStr">
         <is>
-          <t>निकालें</t>
+          <t>बैंक खाता चुनें</t>
         </is>
       </c>
       <c r="F516" t="inlineStr">
         <is>
-          <t>திரும்பப் பெறுக</t>
+          <t>வங்கி கணக்கை தேர்வு செய்யவும்</t>
         </is>
       </c>
       <c r="G516" t="inlineStr">
         <is>
-          <t>ఉపసంహరించుకో</t>
+          <t>బ్యాంకు ఖాతాను ఎంచుకోండి</t>
         </is>
       </c>
     </row>
@@ -19521,32 +19521,32 @@
       </c>
       <c r="B517" t="inlineStr">
         <is>
-          <t>submitting</t>
+          <t>submit</t>
         </is>
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>Withdrawing…</t>
+          <t>Withdraw</t>
         </is>
       </c>
       <c r="D517" t="inlineStr">
         <is>
-          <t>ઉપાડ થઈ રહ્યો છે…</t>
+          <t>ઉપાડ કરો</t>
         </is>
       </c>
       <c r="E517" t="inlineStr">
         <is>
-          <t>निकाला जा रहा है…</t>
+          <t>निकालें</t>
         </is>
       </c>
       <c r="F517" t="inlineStr">
         <is>
-          <t>திரும்பப் பெறுகிறது…</t>
+          <t>திரும்பப் பெறுக</t>
         </is>
       </c>
       <c r="G517" t="inlineStr">
         <is>
-          <t>ఉపసంహరిస్తోంది…</t>
+          <t>ఉపసంహరించుకో</t>
         </is>
       </c>
     </row>
@@ -19558,32 +19558,32 @@
       </c>
       <c r="B518" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>submitting</t>
         </is>
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>Withdraw</t>
+          <t>Withdrawing…</t>
         </is>
       </c>
       <c r="D518" t="inlineStr">
         <is>
-          <t>ઉપાડ</t>
+          <t>ઉપાડ થઈ રહ્યો છે…</t>
         </is>
       </c>
       <c r="E518" t="inlineStr">
         <is>
-          <t>निकासी</t>
+          <t>निकाला जा रहा है…</t>
         </is>
       </c>
       <c r="F518" t="inlineStr">
         <is>
-          <t>திரும்பப் பெறுதல்</t>
+          <t>திரும்பப் பெறுகிறது…</t>
         </is>
       </c>
       <c r="G518" t="inlineStr">
         <is>
-          <t>ఉపసంహరణ</t>
+          <t>ఉపసంహరిస్తోంది…</t>
         </is>
       </c>
     </row>
@@ -19595,32 +19595,32 @@
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>toasts.error</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>Failed to process withdrawal.</t>
+          <t>Withdraw</t>
         </is>
       </c>
       <c r="D519" t="inlineStr">
         <is>
-          <t>ઉપાડ પ્રક્રિયા કરવામાં નિષ્ફળ.</t>
+          <t>ઉપાડ</t>
         </is>
       </c>
       <c r="E519" t="inlineStr">
         <is>
-          <t>निकासी प्रसंस्कृत करने में विफल।</t>
+          <t>निकासी</t>
         </is>
       </c>
       <c r="F519" t="inlineStr">
         <is>
-          <t>திரும்பப் பெறுதலை செயலாக்க தோல்வி.</t>
+          <t>திரும்பப் பெறுதல்</t>
         </is>
       </c>
       <c r="G519" t="inlineStr">
         <is>
-          <t>ఉపసంహరణ ప్రాసెస్ చేయడం విఫలమైంది.</t>
+          <t>ఉపసంహరణ</t>
         </is>
       </c>
     </row>
@@ -19632,32 +19632,32 @@
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>toasts.success</t>
+          <t>toasts.error</t>
         </is>
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>Amount Withdrawal successfully.</t>
+          <t>Failed to process withdrawal.</t>
         </is>
       </c>
       <c r="D520" t="inlineStr">
         <is>
-          <t>રકમ સફળતાપૂર્વક ઉપાડવામાં આવી.</t>
+          <t>ઉપાડ પ્રક્રિયા કરવામાં નિષ્ફળ.</t>
         </is>
       </c>
       <c r="E520" t="inlineStr">
         <is>
-          <t>राशि सफलतापूर्वक निकाली गई।</t>
+          <t>निकासी प्रसंस्कृत करने में विफल।</t>
         </is>
       </c>
       <c r="F520" t="inlineStr">
         <is>
-          <t>தொகை வெற்றிகரமாக திரும்பப் பெறப்பட்டது.</t>
+          <t>திரும்பப் பெறுதலை செயலாக்க தோல்வி.</t>
         </is>
       </c>
       <c r="G520" t="inlineStr">
         <is>
-          <t>మొత్తం విజయవంతంగా ఉపసంహరించబడింది.</t>
+          <t>ఉపసంహరణ ప్రాసెస్ చేయడం విఫలమైంది.</t>
         </is>
       </c>
     </row>
@@ -19669,32 +19669,32 @@
       </c>
       <c r="B521" t="inlineStr">
         <is>
-          <t>validation.amountExceedsMax</t>
+          <t>toasts.success</t>
         </is>
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>You can withdraw a maximum of ₹{{max}}</t>
+          <t>Amount Withdrawal successfully.</t>
         </is>
       </c>
       <c r="D521" t="inlineStr">
         <is>
-          <t>તમે મહત્તમ ₹{{max}} ઉપાડ કરી શકો છો</t>
+          <t>રકમ સફળતાપૂર્વક ઉપાડવામાં આવી.</t>
         </is>
       </c>
       <c r="E521" t="inlineStr">
         <is>
-          <t>आप अधिकतम ₹{{max}} निकाल सकते हैं</t>
+          <t>राशि सफलतापूर्वक निकाली गई।</t>
         </is>
       </c>
       <c r="F521" t="inlineStr">
         <is>
-          <t>அதிகபட்சம் ₹{{max}} திரும்பப் பெறலாம்</t>
+          <t>தொகை வெற்றிகரமாக திரும்பப் பெறப்பட்டது.</t>
         </is>
       </c>
       <c r="G521" t="inlineStr">
         <is>
-          <t>మీరు గరిష్టంగా ₹{{max}} ఉపసంహరించుకోవచ్చు</t>
+          <t>మొత్తం విజయవంతంగా ఉపసంహరించబడింది.</t>
         </is>
       </c>
     </row>
@@ -19706,32 +19706,32 @@
       </c>
       <c r="B522" t="inlineStr">
         <is>
-          <t>validation.amountMinimum</t>
+          <t>validation.amountExceedsMax</t>
         </is>
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>Amount must be greater than ₹500</t>
+          <t>You can withdraw a maximum of ₹{{max}}</t>
         </is>
       </c>
       <c r="D522" t="inlineStr">
         <is>
-          <t>રકમ ₹500 કરતાં વધારે હોવી જોઈએ</t>
+          <t>તમે મહત્તમ ₹{{max}} ઉપાડ કરી શકો છો</t>
         </is>
       </c>
       <c r="E522" t="inlineStr">
         <is>
-          <t>राशि ₹500 से अधिक होनी चाहिए</t>
+          <t>आप अधिकतम ₹{{max}} निकाल सकते हैं</t>
         </is>
       </c>
       <c r="F522" t="inlineStr">
         <is>
-          <t>தொகை ₹500 ஐ விட அதிகமாக இருக்க வேண்டும்</t>
+          <t>அதிகபட்சம் ₹{{max}} திரும்பப் பெறலாம்</t>
         </is>
       </c>
       <c r="G522" t="inlineStr">
         <is>
-          <t>మొత్తం ₹500 కంటే ఎక్కువగా ఉండాలి</t>
+          <t>మీరు గరిష్టంగా ₹{{max}} ఉపసంహరించుకోవచ్చు</t>
         </is>
       </c>
     </row>
@@ -19743,32 +19743,32 @@
       </c>
       <c r="B523" t="inlineStr">
         <is>
-          <t>validation.amountNumbersOnly</t>
+          <t>validation.amountMinimum</t>
         </is>
       </c>
       <c r="C523" t="inlineStr">
         <is>
-          <t>Amount must contain only numbers</t>
+          <t>Amount must be greater than ₹500</t>
         </is>
       </c>
       <c r="D523" t="inlineStr">
         <is>
-          <t>રકમ ફક્ત સંખ્યા ધરાવવી જોઈએ</t>
+          <t>રકમ ₹500 કરતાં વધારે હોવી જોઈએ</t>
         </is>
       </c>
       <c r="E523" t="inlineStr">
         <is>
-          <t>राशि में केवल संख्याएं होनी चाहिए</t>
+          <t>राशि ₹500 से अधिक होनी चाहिए</t>
         </is>
       </c>
       <c r="F523" t="inlineStr">
         <is>
-          <t>தொகையில் எண்கள் மட்டுமே இருக்க வேண்டும்</t>
+          <t>தொகை ₹500 ஐ விட அதிகமாக இருக்க வேண்டும்</t>
         </is>
       </c>
       <c r="G523" t="inlineStr">
         <is>
-          <t>మొత్తంలో సంఖ్యలు మాత్రమే ఉండాలి</t>
+          <t>మొత్తం ₹500 కంటే ఎక్కువగా ఉండాలి</t>
         </is>
       </c>
     </row>
@@ -19780,32 +19780,32 @@
       </c>
       <c r="B524" t="inlineStr">
         <is>
-          <t>validation.amountRequired</t>
+          <t>validation.amountNumbersOnly</t>
         </is>
       </c>
       <c r="C524" t="inlineStr">
         <is>
-          <t>Amount is required</t>
+          <t>Amount must contain only numbers</t>
         </is>
       </c>
       <c r="D524" t="inlineStr">
         <is>
-          <t>રકમ જરૂરી છે</t>
+          <t>રકમ ફક્ત સંખ્યા ધરાવવી જોઈએ</t>
         </is>
       </c>
       <c r="E524" t="inlineStr">
         <is>
-          <t>राशि आवश्यक है</t>
+          <t>राशि में केवल संख्याएं होनी चाहिए</t>
         </is>
       </c>
       <c r="F524" t="inlineStr">
         <is>
-          <t>தொகை தேவை</t>
+          <t>தொகையில் எண்கள் மட்டுமே இருக்க வேண்டும்</t>
         </is>
       </c>
       <c r="G524" t="inlineStr">
         <is>
-          <t>మొత్తం అవసరం</t>
+          <t>మొత్తంలో సంఖ్యలు మాత్రమే ఉండాలి</t>
         </is>
       </c>
     </row>
@@ -19817,32 +19817,32 @@
       </c>
       <c r="B525" t="inlineStr">
         <is>
-          <t>validation.bankRequired</t>
+          <t>validation.amountRequired</t>
         </is>
       </c>
       <c r="C525" t="inlineStr">
         <is>
-          <t>Select Bank Account</t>
+          <t>Amount is required</t>
         </is>
       </c>
       <c r="D525" t="inlineStr">
         <is>
-          <t>બૅન્ક ખાતું પસંદ કરો</t>
+          <t>રકમ જરૂરી છે</t>
         </is>
       </c>
       <c r="E525" t="inlineStr">
         <is>
-          <t>बैंक खाता चुनें</t>
+          <t>राशि आवश्यक है</t>
         </is>
       </c>
       <c r="F525" t="inlineStr">
         <is>
-          <t>வங்கி கணக்கை தேர்வு செய்யவும்</t>
+          <t>தொகை தேவை</t>
         </is>
       </c>
       <c r="G525" t="inlineStr">
         <is>
-          <t>బ్యాంకు ఖాతాను ఎంచుకోండి</t>
+          <t>మొత్తం అవసరం</t>
         </is>
       </c>
     </row>
@@ -19854,32 +19854,32 @@
       </c>
       <c r="B526" t="inlineStr">
         <is>
-          <t>whatsappCta</t>
+          <t>validation.bankRequired</t>
         </is>
       </c>
       <c r="C526" t="inlineStr">
         <is>
-          <t>Withdrawal via WhatsApp</t>
+          <t>Select Bank Account</t>
         </is>
       </c>
       <c r="D526" t="inlineStr">
         <is>
-          <t>WhatsApp દ્વારા ઉપાડ</t>
+          <t>બૅન્ક ખાતું પસંદ કરો</t>
         </is>
       </c>
       <c r="E526" t="inlineStr">
         <is>
-          <t>व्हाट्सऐप के जरिए निकासी</t>
+          <t>बैंक खाता चुनें</t>
         </is>
       </c>
       <c r="F526" t="inlineStr">
         <is>
-          <t>வாட்ஸ்அப் மூலம் திரும்பப் பெறுதல்</t>
+          <t>வங்கி கணக்கை தேர்வு செய்யவும்</t>
         </is>
       </c>
       <c r="G526" t="inlineStr">
         <is>
-          <t>వాట్సాప్ ద్వారా ఉపసంహరణ</t>
+          <t>బ్యాంకు ఖాతాను ఎంచుకోండి</t>
         </is>
       </c>
     </row>
@@ -19891,30 +19891,67 @@
       </c>
       <c r="B527" t="inlineStr">
         <is>
+          <t>whatsappCta</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>Withdrawal via WhatsApp</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>WhatsApp દ્વારા ઉપાડ</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>व्हाट्सऐप के जरिए निकासी</t>
+        </is>
+      </c>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>வாட்ஸ்அப் மூலம் திரும்பப் பெறுதல்</t>
+        </is>
+      </c>
+      <c r="G527" t="inlineStr">
+        <is>
+          <t>వాట్సాప్ ద్వారా ఉపసంహరణ</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>withdraw</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
           <t>withdrawableMoney</t>
         </is>
       </c>
-      <c r="C527" t="inlineStr">
+      <c r="C528" t="inlineStr">
         <is>
           <t>Withdrawal Balance</t>
         </is>
       </c>
-      <c r="D527" t="inlineStr">
+      <c r="D528" t="inlineStr">
         <is>
           <t>ઉપાડ બૅલૅન્સ</t>
         </is>
       </c>
-      <c r="E527" t="inlineStr">
+      <c r="E528" t="inlineStr">
         <is>
           <t>निकासी बैलेंस</t>
         </is>
       </c>
-      <c r="F527" t="inlineStr">
+      <c r="F528" t="inlineStr">
         <is>
           <t>திரும்பப் பெறக்கூடிய இருப்பு</t>
         </is>
       </c>
-      <c r="G527" t="inlineStr">
+      <c r="G528" t="inlineStr">
         <is>
           <t>ఉపసంహరణ బ్యాలెన్స్</t>
         </is>

</xml_diff>